<commit_message>
Télétravail (1 jour par semaine, postes faisables à distance), fermetures ponctuelles de postes, import d'un planning Excel dans Admin
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013i2TqWX3sg1N9rsTKSxB6q
</commit_message>
<xml_diff>
--- a/exemple/parametres_exemple.xlsx
+++ b/exemple/parametres_exemple.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Médecins" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absences" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imposées" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fériés" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fermetures" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fériés" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -243,6 +244,11 @@
     <comment ref="E6" authorId="0" shapeId="0">
       <text>
         <t>Exemple : temps partiel à 80 %.</t>
+      </text>
+    </comment>
+    <comment ref="V8" authorId="0" shapeId="0">
+      <text>
+        <t>Oui = 1 jour de télétravail par semaine (au choix du planning) ; Non = jamais ; « Jeu AM » = seulement le jeudi après-midi.</t>
       </text>
     </comment>
     <comment ref="E11" authorId="0" shapeId="0">
@@ -543,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -621,96 +627,134 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>• Fermetures : postes fermés sur une période (travaux, remplacement de machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>• Fériés : jours non planifiés.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Ajouter un médecin</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Ajoutez une ligne dans l'onglet Médecins (initiales, quotité, off, compétences). Il sera pris en compte à la prochaine génération.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Ajoutez une ligne dans l'onglet Médecins (initiales, quotité, off, compétences). Il sera pris en compte à la prochaine génération.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Pour un ajout ponctuel directement dans un planning déjà généré : voir l'onglet « Lisez-moi » du planning (colonnes libres).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Priorités de couverture (1 = le plus important)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Quand il manque des médecins, les postes de priorité la plus élevée (chiffre le plus grand) ferment en premier.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Quand il manque des médecins, les postes de priorité la plus élevée (chiffre le plus grand) ferment en premier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>La colonne « Priorité au-delà du minimum » s'applique aux places supplémentaires (ex. : 3e médecin au scanner).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Compétences</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Oui = peut tenir le poste · Préféré = affecté en priorité sur ce poste · vide ou Non = jamais affecté.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Codes de demi-journée</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>M = matin, AM = après-midi. Indisponibilités fixes : « Jeu M » ; plusieurs : « Jeu M; Lun AM ».</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>M = matin, AM = après-midi. Indisponibilités fixes : « Jeu M » ; plusieurs : « Jeu M; Lun AM ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Jours off : « Mercredi » ou « Mercredi, Jeudi ». Semaine A / B : alternance une semaine sur deux (voir Paramètres).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Télétravail</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Postes, colonne « Télétravail possible » : Oui pour les postes faisables à distance (scanner, IRM 2…).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Médecins, colonne « Télétravail » : Oui = 1 journée par semaine choisie par le planning ; Non = jamais ; « Jeu AM » = seulement ces demi-journées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Un jour de télétravail, le médecin ne fait que des postes à distance (ex. scanner toute la journée, ou scanner + IRM 2). Il compte dans l'effectif du poste.</t>
         </is>
       </c>
     </row>
@@ -725,7 +769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -900,6 +944,51 @@
       <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Au-delà, le meilleur planning trouvé est retenu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Télétravail : jours par semaine (cible)</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Chaque médecin autorisé (onglet Médecins, colonne Télétravail) a si possible 1 journée par semaine, sur les postes marqués « Oui » dans l'onglet Postes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Télétravail : maximum de jours par semaine</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Au-delà, jamais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Télétravail : maximum de médecins par demi-journée</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Nombre de médecins en télétravail en même temps (0 = sans limite).</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1069,6 +1158,7 @@
     <col width="7" customWidth="1" min="17" max="17"/>
     <col width="7" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1181,6 +1271,11 @@
           <t>Ven AM</t>
         </is>
       </c>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>Télétravail possible</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1268,6 +1363,11 @@
       <c r="S5" s="10" t="inlineStr">
         <is>
           <t>X</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1331,6 +1431,7 @@
       <c r="Q6" s="10" t="inlineStr"/>
       <c r="R6" s="10" t="inlineStr"/>
       <c r="S6" s="10" t="inlineStr"/>
+      <c r="T6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1408,6 +1509,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1461,6 +1563,7 @@
       <c r="Q8" s="10" t="inlineStr"/>
       <c r="R8" s="10" t="inlineStr"/>
       <c r="S8" s="10" t="inlineStr"/>
+      <c r="T8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1546,6 +1649,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1635,6 +1739,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T10" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1720,6 +1829,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1809,6 +1919,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1894,6 +2005,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1983,6 +2095,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -2072,6 +2185,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -2161,6 +2275,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="T16" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2182,7 +2297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U60"/>
+  <dimension ref="A1:V60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2206,6 +2321,7 @@
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2328,6 +2444,11 @@
           <t>BL-RE</t>
         </is>
       </c>
+      <c r="V4" s="7" t="inlineStr">
+        <is>
+          <t>Télétravail</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2405,6 +2526,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V5" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2482,6 +2608,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V6" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2567,6 +2698,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V7" s="10" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2654,6 +2790,11 @@
       <c r="U8" s="10" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="V8" s="10" t="inlineStr">
+        <is>
+          <t>Jeu AM</t>
         </is>
       </c>
     </row>
@@ -2741,6 +2882,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V9" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -2826,6 +2972,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V10" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -2903,6 +3054,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V11" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -2988,6 +3144,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V12" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -3073,6 +3234,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="V13" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -3154,6 +3320,11 @@
       </c>
       <c r="T14" s="10" t="inlineStr"/>
       <c r="U14" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="V14" s="10" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
@@ -3239,6 +3410,11 @@
         </is>
       </c>
       <c r="U15" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="V15" s="10" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
@@ -3266,6 +3442,7 @@
       <c r="S16" s="10" t="inlineStr"/>
       <c r="T16" s="10" t="inlineStr"/>
       <c r="U16" s="10" t="inlineStr"/>
+      <c r="V16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr"/>
@@ -3289,6 +3466,7 @@
       <c r="S17" s="10" t="inlineStr"/>
       <c r="T17" s="10" t="inlineStr"/>
       <c r="U17" s="10" t="inlineStr"/>
+      <c r="V17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr"/>
@@ -3312,6 +3490,7 @@
       <c r="S18" s="10" t="inlineStr"/>
       <c r="T18" s="10" t="inlineStr"/>
       <c r="U18" s="10" t="inlineStr"/>
+      <c r="V18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr"/>
@@ -3335,6 +3514,7 @@
       <c r="S19" s="10" t="inlineStr"/>
       <c r="T19" s="10" t="inlineStr"/>
       <c r="U19" s="10" t="inlineStr"/>
+      <c r="V19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr"/>
@@ -3358,6 +3538,7 @@
       <c r="S20" s="10" t="inlineStr"/>
       <c r="T20" s="10" t="inlineStr"/>
       <c r="U20" s="10" t="inlineStr"/>
+      <c r="V20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr"/>
@@ -3381,6 +3562,7 @@
       <c r="S21" s="10" t="inlineStr"/>
       <c r="T21" s="10" t="inlineStr"/>
       <c r="U21" s="10" t="inlineStr"/>
+      <c r="V21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr"/>
@@ -3404,6 +3586,7 @@
       <c r="S22" s="10" t="inlineStr"/>
       <c r="T22" s="10" t="inlineStr"/>
       <c r="U22" s="10" t="inlineStr"/>
+      <c r="V22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr"/>
@@ -3427,6 +3610,7 @@
       <c r="S23" s="10" t="inlineStr"/>
       <c r="T23" s="10" t="inlineStr"/>
       <c r="U23" s="10" t="inlineStr"/>
+      <c r="V23" s="10" t="inlineStr"/>
     </row>
     <row r="60"/>
   </sheetData>
@@ -4283,6 +4467,353 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Fermetures ponctuelles de postes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Travaux, remplacement de machine… Exemple : IRM1 | 12/10/2026 | 30/10/2026 | Journée | Remplacement de l'IRM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Code poste</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Du</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Période</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Motif</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="9" t="inlineStr"/>
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="9" t="inlineStr"/>
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="10" t="inlineStr"/>
+      <c r="E9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
+      <c r="E10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr"/>
+      <c r="C12" s="9" t="inlineStr"/>
+      <c r="D12" s="10" t="inlineStr"/>
+      <c r="E12" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="9" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="10" t="inlineStr"/>
+      <c r="E13" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr"/>
+      <c r="B14" s="9" t="inlineStr"/>
+      <c r="C14" s="9" t="inlineStr"/>
+      <c r="D14" s="10" t="inlineStr"/>
+      <c r="E14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="9" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="9" t="inlineStr"/>
+      <c r="C16" s="9" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr"/>
+      <c r="E16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr"/>
+      <c r="C17" s="9" t="inlineStr"/>
+      <c r="D17" s="10" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="9" t="inlineStr"/>
+      <c r="C18" s="9" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="9" t="inlineStr"/>
+      <c r="C19" s="9" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr"/>
+      <c r="C20" s="9" t="inlineStr"/>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="9" t="inlineStr"/>
+      <c r="C21" s="9" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="9" t="inlineStr"/>
+      <c r="C22" s="9" t="inlineStr"/>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="9" t="inlineStr"/>
+      <c r="C23" s="9" t="inlineStr"/>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="9" t="inlineStr"/>
+      <c r="C24" s="9" t="inlineStr"/>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="9" t="inlineStr"/>
+      <c r="C25" s="9" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr"/>
+      <c r="E25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+      <c r="B26" s="9" t="inlineStr"/>
+      <c r="C26" s="9" t="inlineStr"/>
+      <c r="D26" s="10" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="9" t="inlineStr"/>
+      <c r="C27" s="9" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr"/>
+      <c r="B28" s="9" t="inlineStr"/>
+      <c r="C28" s="9" t="inlineStr"/>
+      <c r="D28" s="10" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="9" t="inlineStr"/>
+      <c r="C29" s="9" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="9" t="inlineStr"/>
+      <c r="C30" s="9" t="inlineStr"/>
+      <c r="D30" s="10" t="inlineStr"/>
+      <c r="E30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr"/>
+      <c r="B31" s="9" t="inlineStr"/>
+      <c r="C31" s="9" t="inlineStr"/>
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+      <c r="B32" s="9" t="inlineStr"/>
+      <c r="C32" s="9" t="inlineStr"/>
+      <c r="D32" s="10" t="inlineStr"/>
+      <c r="E32" s="10" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr"/>
+      <c r="B33" s="9" t="inlineStr"/>
+      <c r="C33" s="9" t="inlineStr"/>
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr"/>
+      <c r="B34" s="9" t="inlineStr"/>
+      <c r="C34" s="9" t="inlineStr"/>
+      <c r="D34" s="10" t="inlineStr"/>
+      <c r="E34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr"/>
+      <c r="B35" s="9" t="inlineStr"/>
+      <c r="C35" s="9" t="inlineStr"/>
+      <c r="D35" s="10" t="inlineStr"/>
+      <c r="E35" s="10" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr"/>
+      <c r="B36" s="9" t="inlineStr"/>
+      <c r="C36" s="9" t="inlineStr"/>
+      <c r="D36" s="10" t="inlineStr"/>
+      <c r="E36" s="10" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr"/>
+      <c r="B37" s="9" t="inlineStr"/>
+      <c r="C37" s="9" t="inlineStr"/>
+      <c r="D37" s="10" t="inlineStr"/>
+      <c r="E37" s="10" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr"/>
+      <c r="B38" s="9" t="inlineStr"/>
+      <c r="C38" s="9" t="inlineStr"/>
+      <c r="D38" s="10" t="inlineStr"/>
+      <c r="E38" s="10" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr"/>
+      <c r="B39" s="9" t="inlineStr"/>
+      <c r="C39" s="9" t="inlineStr"/>
+      <c r="D39" s="10" t="inlineStr"/>
+      <c r="E39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr"/>
+      <c r="B40" s="9" t="inlineStr"/>
+      <c r="C40" s="9" t="inlineStr"/>
+      <c r="D40" s="10" t="inlineStr"/>
+      <c r="E40" s="10" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr"/>
+      <c r="B41" s="9" t="inlineStr"/>
+      <c r="C41" s="9" t="inlineStr"/>
+      <c r="D41" s="10" t="inlineStr"/>
+      <c r="E41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr"/>
+      <c r="B42" s="9" t="inlineStr"/>
+      <c r="C42" s="9" t="inlineStr"/>
+      <c r="D42" s="10" t="inlineStr"/>
+      <c r="E42" s="10" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr"/>
+      <c r="B43" s="9" t="inlineStr"/>
+      <c r="C43" s="9" t="inlineStr"/>
+      <c r="D43" s="10" t="inlineStr"/>
+      <c r="E43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr"/>
+      <c r="B44" s="9" t="inlineStr"/>
+      <c r="C44" s="9" t="inlineStr"/>
+      <c r="D44" s="10" t="inlineStr"/>
+      <c r="E44" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D5:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Journée,Matin,Après-midi"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Calendrier iPhone dans un onglet dédié ; télétravail limité à 1 médecin par jour, réparti équitablement sur le mois
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013i2TqWX3sg1N9rsTKSxB6q
</commit_message>
<xml_diff>
--- a/exemple/parametres_exemple.xlsx
+++ b/exemple/parametres_exemple.xlsx
@@ -980,7 +980,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Télétravail : maximum de médecins par demi-journée</t>
+          <t>Télétravail : maximum de médecins par jour</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
@@ -988,7 +988,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Nombre de médecins en télétravail en même temps (0 = sans limite).</t>
+          <t>Nombre de médecins en télétravail le même jour (0 = sans limite). Les jours disponibles sont répartis équitablement sur le mois.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Règles du service : ouverture semaine A/B, poste toujours en télétravail, matin/après-midi (interdit, éviter, journée), vacations spécialisées, préférences, notes, astreintes, binôme
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013i2TqWX3sg1N9rsTKSxB6q
</commit_message>
<xml_diff>
--- a/exemple/parametres_exemple.xlsx
+++ b/exemple/parametres_exemple.xlsx
@@ -15,7 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absences" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imposées" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fermetures" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fériés" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vacations spécialisées" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Préférences" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Astreintes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fériés" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -634,31 +638,35 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Fériés : jours non planifiés.</t>
+          <t>• Vacations spécialisées : coro, pédiatrie… tenues par un médecin habilité (obligatoires ou « au moins N par semaine »).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>• Préférences : un médecin plutôt sur un poste ou un site certains jours, ou une demi-journée libre par semaine.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Ajouter un médecin</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>• Notes : réunions et staffs affichés sur le planning (« 1er mardi », « 3e jeudi »…). Astreintes : recopiées depuis l'outil d'astreinte.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Ajoutez une ligne dans l'onglet Médecins (initiales, quotité, off, compétences). Il sera pris en compte à la prochaine génération.</t>
+          <t>• Postes : X = ouvert chaque semaine, A ou B = une semaine sur deux ; « Matin + après-midi » : Interdit, Éviter ou Journée entière ; Télétravail « Toujours » = poste lu à distance uniquement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Pour un ajout ponctuel directement dans un planning déjà généré : voir l'onglet « Lisez-moi » du planning (colonnes libres).</t>
+          <t>• Fériés : jours non planifiés.</t>
         </is>
       </c>
     </row>
@@ -668,21 +676,21 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Priorités de couverture (1 = le plus important)</t>
+          <t>Ajouter un médecin</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Quand il manque des médecins, les postes de priorité la plus élevée (chiffre le plus grand) ferment en premier.</t>
+          <t>Ajoutez une ligne dans l'onglet Médecins (initiales, quotité, off, compétences). Il sera pris en compte à la prochaine génération.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>La colonne « Priorité au-delà du minimum » s'applique aux places supplémentaires (ex. : 3e médecin au scanner).</t>
+          <t>Pour un ajout ponctuel directement dans un planning déjà généré : voir l'onglet « Lisez-moi » du planning (colonnes libres).</t>
         </is>
       </c>
     </row>
@@ -692,38 +700,38 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Compétences</t>
+          <t>Priorités de couverture (1 = le plus important)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Oui = peut tenir le poste · Préféré = affecté en priorité sur ce poste · vide ou Non = jamais affecté.</t>
+          <t>Quand il manque des médecins, les postes de priorité la plus élevée (chiffre le plus grand) ferment en premier.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>La colonne « Priorité au-delà du minimum » s'applique aux places supplémentaires (ex. : 3e médecin au scanner).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Codes de demi-journée</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>M = matin, AM = après-midi. Indisponibilités fixes : « Jeu M » ; plusieurs : « Jeu M; Lun AM ».</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Compétences</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Jours off : « Mercredi » ou « Mercredi, Jeudi ». Semaine A / B : alternance une semaine sur deux (voir Paramètres).</t>
+          <t>Oui = peut tenir le poste · Préféré = affecté en priorité sur ce poste · vide ou Non = jamais affecté.</t>
         </is>
       </c>
     </row>
@@ -733,28 +741,962 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Télétravail</t>
+          <t>Codes de demi-journée</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Onglet Postes, colonne « Télétravail possible » : Oui pour les postes faisables à distance (scanner, IRM 2…).</t>
+          <t>M = matin, AM = après-midi. Indisponibilités fixes : « Jeu M » ; plusieurs : « Jeu M; Lun AM ».</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>Jours off : « Mercredi » ou « Mercredi, Jeudi ». Semaine A / B : alternance une semaine sur deux (voir Paramètres).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Télétravail</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Postes, colonne « Télétravail possible » : Oui pour les postes faisables à distance (scanner, IRM 2…).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>Onglet Médecins, colonne « Télétravail » : Oui = 1 journée par semaine choisie par le planning ; Non = jamais ; « Jeu AM » = seulement ces demi-journées.</t>
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Un jour de télétravail, le médecin ne fait que des postes à distance (ex. scanner toute la journée, ou scanner + IRM 2). Il compte dans l'effectif du poste.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Préférences (souples)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Exemple : OA | Poste | Blaye | Lundi. Ou : SA | Libre | | Mar M, Mar AM (au moins une demi-journée libre).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Médecin</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Poste ou site</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr"/>
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="10" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr"/>
+      <c r="D9" s="10" t="inlineStr"/>
+      <c r="E9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="10" t="inlineStr"/>
+      <c r="C10" s="10" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
+      <c r="E10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr"/>
+      <c r="D12" s="10" t="inlineStr"/>
+      <c r="E12" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr"/>
+      <c r="C13" s="10" t="inlineStr"/>
+      <c r="D13" s="10" t="inlineStr"/>
+      <c r="E13" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr"/>
+      <c r="B14" s="10" t="inlineStr"/>
+      <c r="C14" s="10" t="inlineStr"/>
+      <c r="D14" s="10" t="inlineStr"/>
+      <c r="E14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr"/>
+      <c r="E16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr"/>
+      <c r="D17" s="10" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr"/>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr"/>
+      <c r="C23" s="10" t="inlineStr"/>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr"/>
+      <c r="C24" s="10" t="inlineStr"/>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr"/>
+      <c r="C25" s="10" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr"/>
+      <c r="E25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+      <c r="B26" s="10" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr"/>
+      <c r="D26" s="10" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr"/>
+      <c r="B28" s="10" t="inlineStr"/>
+      <c r="C28" s="10" t="inlineStr"/>
+      <c r="D28" s="10" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr"/>
+      <c r="C30" s="10" t="inlineStr"/>
+      <c r="D30" s="10" t="inlineStr"/>
+      <c r="E30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr"/>
+      <c r="C31" s="10" t="inlineStr"/>
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr"/>
+      <c r="C32" s="10" t="inlineStr"/>
+      <c r="D32" s="10" t="inlineStr"/>
+      <c r="E32" s="10" t="inlineStr"/>
+    </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Un jour de télétravail, le médecin ne fait que des postes à distance (ex. scanner toute la journée, ou scanner + IRM 2). Il compte dans l'effectif du poste.</t>
+      <c r="A33" s="10" t="inlineStr"/>
+      <c r="B33" s="10" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr"/>
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr"/>
+      <c r="C34" s="10" t="inlineStr"/>
+      <c r="D34" s="10" t="inlineStr"/>
+      <c r="E34" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Notes du planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Exemple : Réunion de service 13h30 | 1er mardi. Quand : « 1er mardi », « 3e jeudi », « dernier vendredi », « chaque lundi » ou une date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Quand</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Demi-journée</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="10" t="inlineStr"/>
+      <c r="C10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr"/>
+      <c r="C13" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr"/>
+      <c r="B14" s="10" t="inlineStr"/>
+      <c r="C14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr"/>
+      <c r="C23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr"/>
+      <c r="C24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr"/>
+      <c r="C25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+      <c r="B26" s="10" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr"/>
+      <c r="B28" s="10" t="inlineStr"/>
+      <c r="C28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr"/>
+      <c r="C30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr"/>
+      <c r="C31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr"/>
+      <c r="C32" s="10" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr"/>
+      <c r="B33" s="10" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr"/>
+      <c r="C34" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Astreintes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Recopiées depuis l'outil d'astreinte : une ligne par jour. Le médecin d'astreinte est placé de préférence à l'IRM 1 l'après-midi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Médecin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr"/>
+      <c r="B9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr"/>
+      <c r="B14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr"/>
+      <c r="B26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr"/>
+      <c r="B28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr"/>
+      <c r="B33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr"/>
+      <c r="B35" s="10" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr"/>
+      <c r="B36" s="10" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr"/>
+      <c r="B37" s="10" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr"/>
+      <c r="B38" s="10" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr"/>
+      <c r="B39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr"/>
+      <c r="B40" s="10" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr"/>
+      <c r="B41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr"/>
+      <c r="B42" s="10" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr"/>
+      <c r="B43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr"/>
+      <c r="B44" s="10" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr"/>
+      <c r="B45" s="10" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr"/>
+      <c r="B46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr"/>
+      <c r="B47" s="10" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr"/>
+      <c r="B48" s="10" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr"/>
+      <c r="B49" s="10" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr"/>
+      <c r="B50" s="10" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr"/>
+      <c r="B51" s="10" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr"/>
+      <c r="B52" s="10" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr"/>
+      <c r="B53" s="10" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr"/>
+      <c r="B54" s="10" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr"/>
+      <c r="B55" s="10" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr"/>
+      <c r="B56" s="10" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr"/>
+      <c r="B57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr"/>
+      <c r="B58" s="10" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr"/>
+      <c r="B59" s="10" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr"/>
+      <c r="B60" s="10" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr"/>
+      <c r="B61" s="10" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr"/>
+      <c r="B62" s="10" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr"/>
+      <c r="B63" s="10" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr"/>
+      <c r="B64" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Jours fériés</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Jours non planifiés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Toussaint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>46337</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Armistice</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>46381</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Noël</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>46388</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Jour de l'an</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>46475</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Lundi de Pâques</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>46508</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Fête du travail</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>46513</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Ascension</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>46515</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Victoire 1945</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>46524</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Lundi de Pentecôte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>46582</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Fête nationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>46614</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Assomption</t>
         </is>
       </c>
     </row>
@@ -769,7 +1711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -989,6 +1931,40 @@
       <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Nombre de médecins en télétravail le même jour (0 = sans limite). Les jours disponibles sont répartis équitablement sur le mois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Binôme : jamais absents le même jour</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>IA, IB</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Alerte si les deux sont absents le même jour ; une demande d'absence qui chevauche celle de l'autre est refusée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Binôme : jour de repos de repli</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Si l'un est absent le jour de repos de l'autre, ce repos passe à ce jour-là (salle fermée).</t>
         </is>
       </c>
     </row>
@@ -1136,7 +2112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1159,6 +2135,7 @@
     <col width="7" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1276,6 +2253,11 @@
           <t>Télétravail possible</t>
         </is>
       </c>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>Matin + après-midi</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1370,6 +2352,7 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1432,6 +2415,7 @@
       <c r="R6" s="10" t="inlineStr"/>
       <c r="S6" s="10" t="inlineStr"/>
       <c r="T6" s="10" t="inlineStr"/>
+      <c r="U6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1510,6 +2494,7 @@
         </is>
       </c>
       <c r="T7" s="10" t="inlineStr"/>
+      <c r="U7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1564,6 +2549,7 @@
       <c r="R8" s="10" t="inlineStr"/>
       <c r="S8" s="10" t="inlineStr"/>
       <c r="T8" s="10" t="inlineStr"/>
+      <c r="U8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1650,6 +2636,7 @@
         </is>
       </c>
       <c r="T9" s="10" t="inlineStr"/>
+      <c r="U9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1744,6 +2731,7 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1830,6 +2818,7 @@
         </is>
       </c>
       <c r="T11" s="10" t="inlineStr"/>
+      <c r="U11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1920,6 +2909,7 @@
         </is>
       </c>
       <c r="T12" s="10" t="inlineStr"/>
+      <c r="U12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -2006,6 +2996,7 @@
         </is>
       </c>
       <c r="T13" s="10" t="inlineStr"/>
+      <c r="U13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -2096,6 +3087,7 @@
         </is>
       </c>
       <c r="T14" s="10" t="inlineStr"/>
+      <c r="U14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -2186,6 +3178,7 @@
         </is>
       </c>
       <c r="T15" s="10" t="inlineStr"/>
+      <c r="U15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -2276,11 +3269,18 @@
         </is>
       </c>
       <c r="T16" s="10" t="inlineStr"/>
+      <c r="U16" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="J5:S60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"X"</formula1>
+      <formula1>"X,A,B"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T5:T60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oui,Non,Toujours"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U5:U60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Interdit,Éviter,Journée entière"</formula1>
     </dataValidation>
     <dataValidation sqref="G5:H60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
       <formula1>1</formula1>
@@ -4814,148 +5814,338 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Jours fériés</t>
+          <t>Vacations spécialisées (coro, pédiatrie…)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Jours non planifiés.</t>
+          <t>Exemple : Coro | SCAN | Lun AM, Ven M | SC, DA | 1. Minimum par semaine vide = obligatoire à chaque créneau ; 0 = souhaitée.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Nom</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Libellé</t>
+          <t>Postes</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Créneaux</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Médecins habilités</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Minimum par semaine</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Si présents</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Remarque</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
-        <v>46327</v>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Toussaint</t>
-        </is>
-      </c>
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr"/>
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>46337</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Armistice</t>
-        </is>
-      </c>
+      <c r="A6" s="10" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr"/>
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="10" t="inlineStr"/>
+      <c r="G6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>46381</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Noël</t>
-        </is>
-      </c>
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="10" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>46388</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Jour de l'an</t>
-        </is>
-      </c>
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="10" t="inlineStr"/>
+      <c r="G8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>46475</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Lundi de Pâques</t>
-        </is>
-      </c>
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr"/>
+      <c r="D9" s="10" t="inlineStr"/>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>46508</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Fête du travail</t>
-        </is>
-      </c>
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="10" t="inlineStr"/>
+      <c r="C10" s="10" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
+      <c r="E10" s="10" t="inlineStr"/>
+      <c r="F10" s="10" t="inlineStr"/>
+      <c r="G10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>46513</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Ascension</t>
-        </is>
-      </c>
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="10" t="inlineStr"/>
+      <c r="G11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>46515</v>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Victoire 1945</t>
-        </is>
-      </c>
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr"/>
+      <c r="D12" s="10" t="inlineStr"/>
+      <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="10" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>46524</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Lundi de Pentecôte</t>
-        </is>
-      </c>
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr"/>
+      <c r="C13" s="10" t="inlineStr"/>
+      <c r="D13" s="10" t="inlineStr"/>
+      <c r="E13" s="10" t="inlineStr"/>
+      <c r="F13" s="10" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>46582</v>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Fête nationale</t>
-        </is>
-      </c>
+      <c r="A14" s="10" t="inlineStr"/>
+      <c r="B14" s="10" t="inlineStr"/>
+      <c r="C14" s="10" t="inlineStr"/>
+      <c r="D14" s="10" t="inlineStr"/>
+      <c r="E14" s="10" t="inlineStr"/>
+      <c r="F14" s="10" t="inlineStr"/>
+      <c r="G14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>46614</v>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Assomption</t>
-        </is>
-      </c>
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr"/>
+      <c r="E16" s="10" t="inlineStr"/>
+      <c r="F16" s="10" t="inlineStr"/>
+      <c r="G16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr"/>
+      <c r="D17" s="10" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr"/>
+      <c r="F17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+      <c r="F18" s="10" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr"/>
+      <c r="F19" s="10" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr"/>
+      <c r="G20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr"/>
+      <c r="F21" s="10" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr"/>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr"/>
+      <c r="G22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr"/>
+      <c r="C23" s="10" t="inlineStr"/>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="10" t="inlineStr"/>
+      <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr"/>
+      <c r="C24" s="10" t="inlineStr"/>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr"/>
+      <c r="F24" s="10" t="inlineStr"/>
+      <c r="G24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr"/>
+      <c r="C25" s="10" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr"/>
+      <c r="E25" s="10" t="inlineStr"/>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+      <c r="B26" s="10" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr"/>
+      <c r="D26" s="10" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr"/>
+      <c r="F26" s="10" t="inlineStr"/>
+      <c r="G26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr"/>
+      <c r="F27" s="10" t="inlineStr"/>
+      <c r="G27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr"/>
+      <c r="B28" s="10" t="inlineStr"/>
+      <c r="C28" s="10" t="inlineStr"/>
+      <c r="D28" s="10" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr"/>
+      <c r="F28" s="10" t="inlineStr"/>
+      <c r="G28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr"/>
+      <c r="F29" s="10" t="inlineStr"/>
+      <c r="G29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr"/>
+      <c r="C30" s="10" t="inlineStr"/>
+      <c r="D30" s="10" t="inlineStr"/>
+      <c r="E30" s="10" t="inlineStr"/>
+      <c r="F30" s="10" t="inlineStr"/>
+      <c r="G30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr"/>
+      <c r="C31" s="10" t="inlineStr"/>
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr"/>
+      <c r="F31" s="10" t="inlineStr"/>
+      <c r="G31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr"/>
+      <c r="C32" s="10" t="inlineStr"/>
+      <c r="D32" s="10" t="inlineStr"/>
+      <c r="E32" s="10" t="inlineStr"/>
+      <c r="F32" s="10" t="inlineStr"/>
+      <c r="G32" s="10" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr"/>
+      <c r="B33" s="10" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr"/>
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr"/>
+      <c r="F33" s="10" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr"/>
+      <c r="C34" s="10" t="inlineStr"/>
+      <c r="D34" s="10" t="inlineStr"/>
+      <c r="E34" s="10" t="inlineStr"/>
+      <c r="F34" s="10" t="inlineStr"/>
+      <c r="G34" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>